<commit_message>
Fixed incorrect Zone area inputs
</commit_message>
<xml_diff>
--- a/tests/ExcelLoadData/TieredLoads_Template.xlsx
+++ b/tests/ExcelLoadData/TieredLoads_Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dlvilla\TEMP\TEB\tests\ExcelLoadData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0615404F-0CFD-4093-BABE-77A1B5B11860}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{519F8A7A-14B3-409E-9971-ACA1076DE9AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1905" yWindow="1905" windowWidth="21600" windowHeight="11385" xr2:uid="{1F2B6D78-A821-4296-99B9-3A0B6B938907}"/>
+    <workbookView xWindow="8040" yWindow="8535" windowWidth="21600" windowHeight="11385" xr2:uid="{1F2B6D78-A821-4296-99B9-3A0B6B938907}"/>
   </bookViews>
   <sheets>
     <sheet name="StaticElectricLoads" sheetId="1" r:id="rId1"/>
@@ -707,9 +707,6 @@
     <t>New Name</t>
   </si>
   <si>
-    <t>Per Area (W = False or W/m2 = True?)</t>
-  </si>
-  <si>
     <t>Floor Area (m2)</t>
   </si>
   <si>
@@ -753,6 +750,9 @@
   </si>
   <si>
     <t>Energy (kWh/day or kWh/day/m2)</t>
+  </si>
+  <si>
+    <t>Per Area (kWh = False or kWh/m2 = True?)</t>
   </si>
 </sst>
 </file>
@@ -1212,10 +1212,10 @@
         <v>68</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>107</v>
+        <v>122</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>93</v>
@@ -1224,10 +1224,10 @@
         <v>64</v>
       </c>
       <c r="G1" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="H1" s="2" t="s">
         <v>120</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -54680,7 +54680,7 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B3">
         <v>100</v>
@@ -54694,7 +54694,7 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B4">
         <v>3</v>
@@ -54820,7 +54820,7 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B13">
         <v>0.2</v>
@@ -54834,7 +54834,7 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B14">
         <v>1800</v>
@@ -54848,17 +54848,17 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
@@ -54989,7 +54989,7 @@
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B27">
         <v>0</v>
@@ -55003,7 +55003,7 @@
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="6" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B28">
         <v>0</v>
@@ -55101,7 +55101,7 @@
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" s="6" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B35" t="b">
         <v>1</v>
@@ -55115,7 +55115,7 @@
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" s="6" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B36" t="b">
         <v>1</v>
@@ -55129,7 +55129,7 @@
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B37">
         <v>2.5</v>

</xml_diff>